<commit_message>
Proofread workbook content in British English
</commit_message>
<xml_diff>
--- a/Ecommerce-Stock-and-Order-Control.xlsx
+++ b/Ecommerce-Stock-and-Order-Control.xlsx
@@ -1324,7 +1324,7 @@
         <x:v>6162.5</x:v>
       </x:c>
       <x:c r="F21" s="49" t="str">
-        <x:v>Valid fulfilled revenue</x:v>
+        <x:v>Revenue from valid fulfilled orders</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -8126,7 +8126,7 @@
         <x:v>SKU-012</x:v>
       </x:c>
       <x:c r="E10" s="48" t="str">
-        <x:v>Verify source record and correct before reporting</x:v>
+        <x:v>Verify and correct the source record before reporting.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -8146,7 +8146,7 @@
         <x:v>SKU-019</x:v>
       </x:c>
       <x:c r="E11" s="49" t="str">
-        <x:v>Verify source record and correct before reporting</x:v>
+        <x:v>Verify and correct the source record before reporting.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -8166,7 +8166,7 @@
         <x:v>SKU-999</x:v>
       </x:c>
       <x:c r="E12" s="49" t="str">
-        <x:v>Verify source record and correct before reporting</x:v>
+        <x:v>Verify and correct the source record before reporting.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -8186,7 +8186,7 @@
         <x:v>SKU-034</x:v>
       </x:c>
       <x:c r="E13" s="49" t="str">
-        <x:v>Verify source record and correct before reporting</x:v>
+        <x:v>Verify and correct the source record before reporting.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -8206,7 +8206,7 @@
         <x:v>SKU-019</x:v>
       </x:c>
       <x:c r="E14" s="49" t="str">
-        <x:v>Verify source record and correct before reporting</x:v>
+        <x:v>Verify and correct the source record before reporting.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">

</xml_diff>